<commit_message>
Remove bad issues, fix specs, improve prompt
</commit_message>
<xml_diff>
--- a/Issues_No_Tests_v1.xlsx
+++ b/Issues_No_Tests_v1.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:M36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -516,21 +516,21 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>648</v>
+        <v>4717</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>[Feature Request] Implement Double-band EAM Potential Style</t>
+          <t>[BUG] _Inconsistencies in dipolar energy between spin/dipole/long and spin/dipole/cut pair styles_</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/648</t>
+          <t>https://github.com/lammps/lammps/issues/4717</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -541,18 +541,16 @@
       <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>enhancement
-manybody_package
-volunteer_needed</t>
+          <t>bug</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/5039</t>
+          <t>https://github.com/lammps/lammps/pull/5042</t>
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>5039</v>
+        <v>5042</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -562,7 +560,7 @@
       <c r="L2" s="3" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>The issue requests implementation of a double-band EAM potential style, referencing specific physics/materials science formalism (two-band EAM, s- and d-electron contributions) from scientific papers, which requires domain-specific knowledge to implement.</t>
+          <t>The issue reports incorrect dipolar energy calculations between pair styles, requiring analytical dipolar formulas and spin configurations, and includes attached PDF plots of the test results.</t>
         </is>
       </c>
     </row>
@@ -573,21 +571,21 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>4717</v>
+        <v>4855</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>[BUG] _Inconsistencies in dipolar energy between spin/dipole/long and spin/dipole/cut pair styles_</t>
+          <t>Inconsistent behavior of the GPU-accelerated CORE-SHELL model</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4717</t>
+          <t>https://github.com/lammps/lammps/issues/4855</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>1,2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -603,11 +601,11 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/5042</t>
+          <t>https://github.com/lammps/lammps/pull/4887</t>
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>5042</v>
+        <v>4887</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -617,7 +615,7 @@
       <c r="L3" s="3" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>The issue reports incorrect dipolar energy calculations between pair styles, requiring analytical dipolar formulas and spin configurations, and includes attached PDF plots of the test results.</t>
+          <t>The issue concerns inconsistent physics of the GPU-accelerated core-shell model, involving Coulomb/Ewald sums, cutoff dependence, lattice parameters, and phase transition temperatures, which requires domain-specific scientific knowledge to understand.</t>
         </is>
       </c>
     </row>
@@ -628,29 +626,34 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>4855</v>
+        <v>4602</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Inconsistent behavior of the GPU-accelerated CORE-SHELL model</t>
+          <t>[BUG] Velocity profiles with fix srd and fix deform shear flow</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4855</t>
+          <t>https://github.com/lammps/lammps/issues/4602</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/user-attachments/assets/d01d6ffb-cb4c-4fbf-9746-90fc3afc0d0b
+https://github.com/user-attachments/assets/c56fb6b5-15cd-4114-88d9-1d11fdd4bbef</t>
+        </is>
+      </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
           <t>bug</t>
@@ -658,11 +661,11 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4887</t>
+          <t>https://github.com/lammps/lammps/pull/4590</t>
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>4887</v>
+        <v>4590</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -672,7 +675,7 @@
       <c r="L4" s="3" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>The issue concerns inconsistent physics of the GPU-accelerated core-shell model, involving Coulomb/Ewald sums, cutoff dependence, lattice parameters, and phase transition temperatures, which requires domain-specific scientific knowledge to understand.</t>
+          <t>The issue describes incorrect scientific behavior in SRD shear flow simulation with fix deform and fix srd, and includes scientific velocity profile plots showing the kink and vanishing profile.</t>
         </is>
       </c>
     </row>
@@ -683,21 +686,21 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>4602</v>
+        <v>4770</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>[BUG] Velocity profiles with fix srd and fix deform shear flow</t>
+          <t>[BUG] Incorrect kernel gradients in ComputeRHEOVShift::correct_type_interface()</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4602</t>
+          <t>https://github.com/lammps/lammps/issues/4770</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>1,2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -707,8 +710,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/user-attachments/assets/d01d6ffb-cb4c-4fbf-9746-90fc3afc0d0b
-https://github.com/user-attachments/assets/c56fb6b5-15cd-4114-88d9-1d11fdd4bbef</t>
+          <t>https://github.com/user-attachments/assets/404cd62f-9100-4445-8764-bd8380b67942</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -718,11 +720,11 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4590</t>
+          <t>https://github.com/lammps/lammps/pull/4861</t>
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>4590</v>
+        <v>4861</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
@@ -732,7 +734,7 @@
       <c r="L5" s="3" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>The issue describes incorrect scientific behavior in SRD shear flow simulation with fix deform and fix srd, and includes scientific velocity profile plots showing the kink and vanishing profile.</t>
+          <t>The issue reports incorrect SPH kernel gradient calculations and discusses color function/proportion formulations for phase interface identification, involving domain-specific scientific equations and numerical methods.</t>
         </is>
       </c>
     </row>
@@ -743,16 +745,16 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>4770</v>
+        <v>4767</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>[BUG] Incorrect kernel gradients in ComputeRHEOVShift::correct_type_interface()</t>
+          <t>[BUG] Incorrect forces in fix/langevin/kk due to velocity update overwriting in non-Kokkos compute/temp/com</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4770</t>
+          <t>https://github.com/lammps/lammps/issues/4767</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -762,26 +764,23 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>https://github.com/user-attachments/assets/404cd62f-9100-4445-8764-bd8380b67942</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>bug</t>
+          <t>bug
+kokkos_package</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4861</t>
+          <t>https://github.com/lammps/lammps/pull/4768</t>
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>4861</v>
+        <v>4768</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
@@ -791,7 +790,7 @@
       <c r="L6" s="3" t="inlineStr"/>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>The issue reports incorrect SPH kernel gradient calculations and discusses color function/proportion formulations for phase interface identification, involving domain-specific scientific equations and numerical methods.</t>
+          <t>The bug involves incorrect Langevin thermostat force calculations due to velocity updates, which is domain-specific scientific/physics content.</t>
         </is>
       </c>
     </row>
@@ -802,16 +801,16 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>4767</v>
+        <v>4679</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>[BUG] Incorrect forces in fix/langevin/kk due to velocity update overwriting in non-Kokkos compute/temp/com</t>
+          <t>[Feature Request] _fix SHAKE force constraint</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4767</t>
+          <t>https://github.com/lammps/lammps/issues/4679</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -827,17 +826,16 @@
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>bug
-kokkos_package</t>
+          <t>enhancement</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4768</t>
+          <t>https://github.com/lammps/lammps/pull/4760</t>
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>4768</v>
+        <v>4760</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
@@ -847,7 +845,7 @@
       <c r="L7" s="3" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>The bug involves incorrect Langevin thermostat force calculations due to velocity updates, which is domain-specific scientific/physics content.</t>
+          <t>The issue requests access to SHAKE constraint forces for computing potential mean force, which involves domain-specific molecular dynamics and constrained-bond scientific concepts.</t>
         </is>
       </c>
     </row>
@@ -858,16 +856,16 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>4679</v>
+        <v>4726</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>[Feature Request] _fix SHAKE force constraint</t>
+          <t>[BUG] Molecule JSON vs .molecule_template molecule command parsing causes different simulation outputs</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4679</t>
+          <t>https://github.com/lammps/lammps/issues/4726</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -883,16 +881,16 @@
       <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>enhancement</t>
+          <t>bug</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4760</t>
+          <t>https://github.com/lammps/lammps/pull/4732</t>
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>4760</v>
+        <v>4732</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
@@ -902,7 +900,7 @@
       <c r="L8" s="3" t="inlineStr"/>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>The issue requests access to SHAKE constraint forces for computing potential mean force, which involves domain-specific molecular dynamics and constrained-bond scientific concepts.</t>
+          <t>The issue describes differing simulation outputs for equivalent molecule files, involving reaction progress and molecular topology in LAMMPS, which is domain-specific scientific behavior.</t>
         </is>
       </c>
     </row>
@@ -913,16 +911,16 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>4726</v>
+        <v>565</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>[BUG] Molecule JSON vs .molecule_template molecule command parsing causes different simulation outputs</t>
+          <t>[Feature Request] hybrid monte carlo</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4726</t>
+          <t>https://github.com/lammps/lammps/issues/565</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -937,123 +935,123 @@
       </c>
       <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>bug</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>https://github.com/lammps/lammps/pull/4732</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="n">
-        <v>4732</v>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L9" s="3" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr">
-        <is>
-          <t>The issue describes differing simulation outputs for equivalent molecule files, involving reaction progress and molecular topology in LAMMPS, which is domain-specific scientific behavior.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>lammps/lammps</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>565</v>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>[Feature Request] hybrid monte carlo</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>https://github.com/lammps/lammps/issues/565</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr"/>
-      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>enhancement
 mc_package
 volunteer_needed</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>https://github.com/lammps/lammps/pull/4019</t>
         </is>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="J9" s="2" t="n">
         <v>4019</v>
       </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L10" s="3" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr"/>
+      <c r="M9" s="3" t="inlineStr">
         <is>
           <t>The issue requests implementation of Hybrid Monte Carlo simulations, discussing detailed balance, acceptance/rejection of MD moves, and velocity re-randomization, which are domain-specific scientific and algorithmic concepts.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>lammps/lammps</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>lammps/lammps</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
         <v>4568</v>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>A possible bug in RHEO/compute_rheo_interface.cpp</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>https://github.com/lammps/lammps/issues/4568</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>https://github.com/user-attachments/assets/f383e4dc-ee20-4152-ad09-6058b3fbd8b7
 https://github.com/user-attachments/assets/2242b093-3b6e-4480-95f8-3a0c4410bafb
 https://github.com/user-attachments/assets/b1c98fa3-af6c-469d-8e30-b7674158f161</t>
         </is>
       </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/lammps/lammps/pull/4545</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>4545</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr"/>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>The issue discusses the incorrect implementation of a density lower limit rho0/10 in a fluid-solid interaction model, requiring domain knowledge of the RHEO method and physical unit systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>lammps/lammps</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>4491</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>[BUG] _Wrong coordination number (CN) with compute rdf</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/lammps/lammps/issues/4491</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
       <c r="H11" s="3" t="inlineStr">
         <is>
           <t>bug</t>
@@ -1061,11 +1059,11 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4545</t>
+          <t>https://github.com/lammps/lammps/pull/4481</t>
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>4545</v>
+        <v>4481</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
@@ -1075,7 +1073,7 @@
       <c r="L11" s="3" t="inlineStr"/>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>The issue discusses the incorrect implementation of a density lower limit rho0/10 in a fluid-solid interaction model, requiring domain knowledge of the RHEO method and physical unit systems.</t>
+          <t>The bug concerns incorrect coordination numbers from a radial distribution function calculation, which requires understanding of chemistry/domain-specific scientific concepts like coordination number and RDF.</t>
         </is>
       </c>
     </row>
@@ -1086,16 +1084,16 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>4491</v>
+        <v>2017</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>[BUG] _Wrong coordination number (CN) with compute rdf</t>
+          <t>[BUG] Gay-Berne pair style does not honour special-bonds in the GPU package</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4491</t>
+          <t>https://github.com/lammps/lammps/issues/2017</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1116,11 +1114,11 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4481</t>
+          <t>https://github.com/lammps/lammps/pull/2026</t>
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>4481</v>
+        <v>2026</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
@@ -1130,7 +1128,7 @@
       <c r="L12" s="3" t="inlineStr"/>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>The bug concerns incorrect coordination numbers from a radial distribution function calculation, which requires understanding of chemistry/domain-specific scientific concepts like coordination number and RDF.</t>
+          <t>The bug concerns incorrect computation of Gay-Berne interactions for special-bonded pairs, involving molecular simulation force-field behavior and incorrect energy/force/torque results, which requires domain-specific scientific knowledge to assess.</t>
         </is>
       </c>
     </row>
@@ -1141,16 +1139,16 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>2017</v>
+        <v>1657</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>[BUG] Gay-Berne pair style does not honour special-bonds in the GPU package</t>
+          <t>[BUG] No rigid body rotation for rigid/nve styles</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/2017</t>
+          <t>https://github.com/lammps/lammps/issues/1657</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1166,16 +1164,17 @@
       <c r="G13" s="3" t="inlineStr"/>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>bug</t>
+          <t>bug
+documentation</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/2026</t>
+          <t>https://github.com/lammps/lammps/pull/2105</t>
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>2026</v>
+        <v>2105</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
@@ -1185,7 +1184,7 @@
       <c r="L13" s="3" t="inlineStr"/>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>The bug concerns incorrect computation of Gay-Berne interactions for special-bonded pairs, involving molecular simulation force-field behavior and incorrect energy/force/torque results, which requires domain-specific scientific knowledge to assess.</t>
+          <t>The issue concerns missing rotational dynamics of granular rigid bodies in LAMMPS, involving physical concepts such as moments of inertia, units, and rigid-body motion.</t>
         </is>
       </c>
     </row>
@@ -1196,16 +1195,16 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>1657</v>
+        <v>2288</v>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>[BUG] No rigid body rotation for rigid/nve styles</t>
+          <t>[BUG] fix rigid/nve langevin not working as expected</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/1657</t>
+          <t>https://github.com/lammps/lammps/issues/2288</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1221,17 +1220,16 @@
       <c r="G14" s="3" t="inlineStr"/>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>bug
-documentation</t>
+          <t>bug</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/2105</t>
+          <t>https://github.com/lammps/lammps/pull/2367</t>
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>2105</v>
+        <v>2367</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
@@ -1241,7 +1239,7 @@
       <c r="L14" s="3" t="inlineStr"/>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>The issue concerns missing rotational dynamics of granular rigid bodies in LAMMPS, involving physical concepts such as moments of inertia, units, and rigid-body motion.</t>
+          <t>The issue concerns incorrect thermodynamic behavior of a Langevin thermostat in molecular dynamics simulations, involving kinetic energy, temperature control, and degrees of freedom of rigid molecules.</t>
         </is>
       </c>
     </row>
@@ -1252,16 +1250,16 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>2288</v>
+        <v>4398</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>[BUG] fix rigid/nve langevin not working as expected</t>
+          <t>[BUG] Incorrect centre of mass with fix reaxff/species position option</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/2288</t>
+          <t>https://github.com/lammps/lammps/issues/4398</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1282,11 +1280,11 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/2367</t>
+          <t>https://github.com/lammps/lammps/pull/4443</t>
         </is>
       </c>
       <c r="J15" s="2" t="n">
-        <v>2367</v>
+        <v>4443</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
@@ -1296,7 +1294,7 @@
       <c r="L15" s="3" t="inlineStr"/>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>The issue concerns incorrect thermodynamic behavior of a Langevin thermostat in molecular dynamics simulations, involving kinetic energy, temperature control, and degrees of freedom of rigid molecules.</t>
+          <t>The issue reports incorrect scientific output from fix reaxff/species, specifically average atomic positions and average charge being reported instead of center-of-mass positions and total charge, which involves domain-specific physical/chemical concepts.</t>
         </is>
       </c>
     </row>
@@ -1307,84 +1305,29 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>4398</v>
+        <v>4306</v>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>[BUG] Incorrect centre of mass with fix reaxff/species position option</t>
+          <t>[Feature Request] Add angleoffset for hbond/dreiding/morse and hbond/dreiding/lj</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4398</t>
+          <t>https://github.com/lammps/lammps/issues/4306</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr"/>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>bug</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>https://github.com/lammps/lammps/pull/4443</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="n">
-        <v>4443</v>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L16" s="3" t="inlineStr"/>
-      <c r="M16" s="3" t="inlineStr">
-        <is>
-          <t>The issue reports incorrect scientific output from fix reaxff/species, specifically average atomic positions and average charge being reported instead of center-of-mass positions and total charge, which involves domain-specific physical/chemical concepts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>lammps/lammps</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>4306</v>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>[Feature Request] Add angleoffset for hbond/dreiding/morse and hbond/dreiding/lj</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>https://github.com/lammps/lammps/issues/4306</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>1,2</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>https://docs.lammps.org/_images/dreiding_hbond.jpg
 https://github.com/user-attachments/assets/b0a66bd2-e3d9-4d50-9c73-172eba8ef979
@@ -1392,6 +1335,61 @@
 https://github.com/user-attachments/assets/936c999d-6fc4-435f-b4e3-d0c6fe61cee2</t>
         </is>
       </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/lammps/lammps/pull/4310</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>4310</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr"/>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>The issue involves molecular geometry and hydrogen bonding angle math (adding an angle offset to the hbond/dreiding potential) and includes a scientific image of the hydrogen bond geometry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>lammps/lammps</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>4226</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>[Feature Request] Allow for QTPIE charge equilibration with external efield</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/lammps/lammps/issues/4226</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr"/>
       <c r="H17" s="3" t="inlineStr">
         <is>
           <t>enhancement</t>
@@ -1399,11 +1397,11 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4310</t>
+          <t>https://github.com/lammps/lammps/pull/4312</t>
         </is>
       </c>
       <c r="J17" s="2" t="n">
-        <v>4310</v>
+        <v>4312</v>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
@@ -1413,7 +1411,7 @@
       <c r="L17" s="3" t="inlineStr"/>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>The issue involves molecular geometry and hydrogen bonding angle math (adding an angle offset to the hbond/dreiding potential) and includes a scientific image of the hydrogen bond geometry.</t>
+          <t>The issue discusses implementing QTPIE charge equilibration with external electric fields, involving electronegativity equations, unit conversions for electric field terms, and domain-specific chemistry/physics concepts.</t>
         </is>
       </c>
     </row>
@@ -1424,16 +1422,16 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>4226</v>
+        <v>4219</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>[Feature Request] Allow for QTPIE charge equilibration with external efield</t>
+          <t>[BUG] _Wrong forces input for bulk stress tensor calculation in pair granular/hooke/history/kk_</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4226</t>
+          <t>https://github.com/lammps/lammps/issues/4219</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1449,16 +1447,16 @@
       <c r="G18" s="3" t="inlineStr"/>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>enhancement</t>
+          <t>bug</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4312</t>
+          <t>https://github.com/lammps/lammps/pull/4346</t>
         </is>
       </c>
       <c r="J18" s="2" t="n">
-        <v>4312</v>
+        <v>4346</v>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
@@ -1468,7 +1466,7 @@
       <c r="L18" s="3" t="inlineStr"/>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>The issue discusses implementing QTPIE charge equilibration with external electric fields, involving electronegativity equations, unit conversions for electric field terms, and domain-specific chemistry/physics concepts.</t>
+          <t>The issue describes incorrect stress tensor calculation in a granular simulation, involving physical concepts of forces and stress, which is a scientific correctness bug in the numerical method.</t>
         </is>
       </c>
     </row>
@@ -1479,16 +1477,16 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>4219</v>
+        <v>4337</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>[BUG] _Wrong forces input for bulk stress tensor calculation in pair granular/hooke/history/kk_</t>
+          <t>[BUG]  GRANULAR package fix_pour:  wrong insertion volume calculation (particularly in in SI units)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4219</t>
+          <t>https://github.com/lammps/lammps/issues/4337</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1509,11 +1507,11 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4346</t>
+          <t>https://github.com/lammps/lammps/pull/4339</t>
         </is>
       </c>
       <c r="J19" s="2" t="n">
-        <v>4346</v>
+        <v>4339</v>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
@@ -1523,7 +1521,7 @@
       <c r="L19" s="3" t="inlineStr"/>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>The issue describes incorrect stress tensor calculation in a granular simulation, involving physical concepts of forces and stress, which is a scientific correctness bug in the numerical method.</t>
+          <t>The bug concerns incorrect physical volume calculation for particle insertion in granular simulations, which requires scientific/domain knowledge of units and geometry.</t>
         </is>
       </c>
     </row>
@@ -1534,16 +1532,16 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>4337</v>
+        <v>3831</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>[BUG]  GRANULAR package fix_pour:  wrong insertion volume calculation (particularly in in SI units)</t>
+          <t>[BUG] SPH/DPD packages incompatible with velocity remapping</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4337</t>
+          <t>https://github.com/lammps/lammps/issues/3831</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1559,16 +1557,17 @@
       <c r="G20" s="3" t="inlineStr"/>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>bug</t>
+          <t>bug
+user_dpd_package</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4339</t>
+          <t>https://github.com/lammps/lammps/pull/4243</t>
         </is>
       </c>
       <c r="J20" s="2" t="n">
-        <v>4339</v>
+        <v>4243</v>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
@@ -1578,7 +1577,7 @@
       <c r="L20" s="3" t="inlineStr"/>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>The bug concerns incorrect physical volume calculation for particle insertion in granular simulations, which requires scientific/domain knowledge of units and geometry.</t>
+          <t>The issue describes incorrect physics in SPH/DPD simulations due to missing velocity remapping terms under shear, involving domain-specific knowledge of periodic boundaries and velocity extrapolation.</t>
         </is>
       </c>
     </row>
@@ -1589,16 +1588,16 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>3831</v>
+        <v>4231</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>[BUG] SPH/DPD packages incompatible with velocity remapping</t>
+          <t>[BUG] Wrong CNA value(and neighbor list) when LAMMPS is run in a loop using next</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/3831</t>
+          <t>https://github.com/lammps/lammps/issues/4231</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1614,17 +1613,16 @@
       <c r="G21" s="3" t="inlineStr"/>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>bug
-user_dpd_package</t>
+          <t>bug</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4243</t>
+          <t>https://github.com/lammps/lammps/pull/4239</t>
         </is>
       </c>
       <c r="J21" s="2" t="n">
-        <v>4243</v>
+        <v>4239</v>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
@@ -1634,7 +1632,7 @@
       <c r="L21" s="3" t="inlineStr"/>
       <c r="M21" s="3" t="inlineStr">
         <is>
-          <t>The issue describes incorrect physics in SPH/DPD simulations due to missing velocity remapping terms under shear, involving domain-specific knowledge of periodic boundaries and velocity extrapolation.</t>
+          <t>The bug concerns incorrect Common Neighbor Analysis (CNA) values, which is a domain-specific crystallography/materials-science algorithm and incorrect scientific output.</t>
         </is>
       </c>
     </row>
@@ -1645,16 +1643,16 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>4216</v>
+        <v>4153</v>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>[BUG] _fix nonaffine/displacement not work in rerun</t>
+          <t>[BUG] Incorrect output for triclinic/general when using dump style custom</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4216</t>
+          <t>https://github.com/lammps/lammps/issues/4153</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1675,11 +1673,11 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4339</t>
+          <t>https://github.com/lammps/lammps/pull/4202</t>
         </is>
       </c>
       <c r="J22" s="2" t="n">
-        <v>4339</v>
+        <v>4202</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
@@ -1689,7 +1687,7 @@
       <c r="L22" s="3" t="inlineStr"/>
       <c r="M22" s="3" t="inlineStr">
         <is>
-          <t>The issue involves incorrect results from the nonaffine/displacement calculation, a domain-specific scientific analysis in molecular dynamics, and thus requires understanding of that physical concept.</t>
+          <t>The bug concerns incorrect transformation of atomic positions and simulation cell vectors for triclinic systems in LAMMPS dump output, which involves domain-specific scientific concepts of lattice geometry and molecular simulation coordinate representation.</t>
         </is>
       </c>
     </row>
@@ -1700,16 +1698,16 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>4231</v>
+        <v>4141</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>[BUG] Wrong CNA value(and neighbor list) when LAMMPS is run in a loop using next</t>
+          <t>[BUG] Inconsistency using fix wall/gran with the granular pairstyle</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4231</t>
+          <t>https://github.com/lammps/lammps/issues/4141</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1725,16 +1723,17 @@
       <c r="G23" s="3" t="inlineStr"/>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>bug</t>
+          <t>bug
+granular_package</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4239</t>
+          <t>https://github.com/lammps/lammps/pull/4195</t>
         </is>
       </c>
       <c r="J23" s="2" t="n">
-        <v>4239</v>
+        <v>4195</v>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
@@ -1744,7 +1743,7 @@
       <c r="L23" s="3" t="inlineStr"/>
       <c r="M23" s="3" t="inlineStr">
         <is>
-          <t>The bug concerns incorrect Common Neighbor Analysis (CNA) values, which is a domain-specific crystallography/materials-science algorithm and incorrect scientific output.</t>
+          <t>The issue describes incorrect physical behavior in Hertzian granular contact mechanics, specifically the effective Young's modulus mixing rule for particle-wall interactions, which requires domain-specific scientific knowledge to understand.</t>
         </is>
       </c>
     </row>
@@ -1755,16 +1754,16 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>4153</v>
+        <v>4180</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>[BUG] Incorrect output for triclinic/general when using dump style custom</t>
+          <t>[BUG] Cohesion + damping `coeff_restitution` can result in nan positions</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4153</t>
+          <t>https://github.com/lammps/lammps/issues/4180</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1785,11 +1784,11 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4202</t>
+          <t>https://github.com/lammps/lammps/pull/4195</t>
         </is>
       </c>
       <c r="J24" s="2" t="n">
-        <v>4202</v>
+        <v>4195</v>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
@@ -1799,7 +1798,7 @@
       <c r="L24" s="3" t="inlineStr"/>
       <c r="M24" s="3" t="inlineStr">
         <is>
-          <t>The bug concerns incorrect transformation of atomic positions and simulation cell vectors for triclinic systems in LAMMPS dump output, which involves domain-specific scientific concepts of lattice geometry and molecular simulation coordinate representation.</t>
+          <t>The issue involves incorrect mathematical formulation of the damping coefficient in cohesive DMT contact models, referencing equations and physical constants that lead to nan positions.</t>
         </is>
       </c>
     </row>
@@ -1810,16 +1809,16 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>4141</v>
+        <v>3982</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>[BUG] Inconsistency using fix wall/gran with the granular pairstyle</t>
+          <t>documentation and/or error handling for eam/alloy</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4141</t>
+          <t>https://github.com/lammps/lammps/issues/3982</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1833,19 +1832,14 @@
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>bug
-granular_package</t>
-        </is>
-      </c>
+      <c r="H25" s="3" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4195</t>
+          <t>https://github.com/lammps/lammps/pull/4134</t>
         </is>
       </c>
       <c r="J25" s="2" t="n">
-        <v>4195</v>
+        <v>4134</v>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
@@ -1855,7 +1849,7 @@
       <c r="L25" s="3" t="inlineStr"/>
       <c r="M25" s="3" t="inlineStr">
         <is>
-          <t>The issue describes incorrect physical behavior in Hertzian granular contact mechanics, specifically the effective Young's modulus mixing rule for particle-wall interactions, which requires domain-specific scientific knowledge to understand.</t>
+          <t>The issue discusses EAM potential behavior with electron density exceeding the tabulated maximum, involving embedding energy and scientific domain knowledge about interatomic potentials.</t>
         </is>
       </c>
     </row>
@@ -1866,16 +1860,16 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>4180</v>
+        <v>4109</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>[BUG] Cohesion + damping `coeff_restitution` can result in nan positions</t>
+          <t>[BUG] _Unable to restart from restart files with rigid molecules.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4180</t>
+          <t>https://github.com/lammps/lammps/issues/4109</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1896,11 +1890,11 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4195</t>
+          <t>https://github.com/lammps/lammps/pull/4123</t>
         </is>
       </c>
       <c r="J26" s="2" t="n">
-        <v>4195</v>
+        <v>4123</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
@@ -1910,7 +1904,7 @@
       <c r="L26" s="3" t="inlineStr"/>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t>The issue involves incorrect mathematical formulation of the damping coefficient in cohesive DMT contact models, referencing equations and physical constants that lead to nan positions.</t>
+          <t>The issue involves molecular dynamics simulation concepts such as rigid molecules, periodic boundary conditions, and minimum image conventions, which are necessary to understand the restart failure.</t>
         </is>
       </c>
     </row>
@@ -1921,16 +1915,16 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>3982</v>
+        <v>4119</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>documentation and/or error handling for eam/alloy</t>
+          <t>[BUG] pair_style ylz needs explicit symmetrization of the interaction cutoff</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/3982</t>
+          <t>https://github.com/lammps/lammps/issues/4119</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1944,14 +1938,18 @@
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr"/>
-      <c r="H27" s="3" t="inlineStr"/>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4134</t>
+          <t>https://github.com/lammps/lammps/pull/4120</t>
         </is>
       </c>
       <c r="J27" s="2" t="n">
-        <v>4134</v>
+        <v>4120</v>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
@@ -1961,7 +1959,7 @@
       <c r="L27" s="3" t="inlineStr"/>
       <c r="M27" s="3" t="inlineStr">
         <is>
-          <t>The issue discusses EAM potential behavior with electron density exceeding the tabulated maximum, involving embedding energy and scientific domain knowledge about interatomic potentials.</t>
+          <t>The issue describes incorrect force calculations and differing MD trajectories due to improper handling of pair style coefficients and cutoff symmetrization, which is domain-specific scientific behavior in molecular dynamics simulations.</t>
         </is>
       </c>
     </row>
@@ -1972,16 +1970,16 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>4109</v>
+        <v>3545</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>[BUG] _Unable to restart from restart files with rigid molecules.</t>
+          <t>[BUG] Wrong delxyz calculation in region_ellipsoid.cpp</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4109</t>
+          <t>https://github.com/lammps/lammps/issues/3545</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2002,11 +2000,11 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4123</t>
+          <t>https://github.com/lammps/lammps/pull/3553</t>
         </is>
       </c>
       <c r="J28" s="2" t="n">
-        <v>4123</v>
+        <v>3553</v>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
@@ -2016,7 +2014,7 @@
       <c r="L28" s="3" t="inlineStr"/>
       <c r="M28" s="3" t="inlineStr">
         <is>
-          <t>The issue involves molecular dynamics simulation concepts such as rigid molecules, periodic boundary conditions, and minimum image conventions, which are necessary to understand the restart failure.</t>
+          <t>The issue reports incorrect vector calculations in ellipsoid region surface code, involving mathematical formulas for contact distance vectors that are necessary to understand the bug.</t>
         </is>
       </c>
     </row>
@@ -2027,16 +2025,16 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>4119</v>
+        <v>3925</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>[BUG] pair_style ylz needs explicit symmetrization of the interaction cutoff</t>
+          <t>[BUG] fix wall/region with region style ellipsoid</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4119</t>
+          <t>https://github.com/lammps/lammps/issues/3925</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2057,11 +2055,11 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4120</t>
+          <t>https://github.com/lammps/lammps/pull/3931</t>
         </is>
       </c>
       <c r="J29" s="2" t="n">
-        <v>4120</v>
+        <v>3931</v>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
@@ -2071,7 +2069,7 @@
       <c r="L29" s="3" t="inlineStr"/>
       <c r="M29" s="3" t="inlineStr">
         <is>
-          <t>The issue describes incorrect force calculations and differing MD trajectories due to improper handling of pair style coefficients and cutoff symmetrization, which is domain-specific scientific behavior in molecular dynamics simulations.</t>
+          <t>The bug involves incorrect mathematical formulas for the ellipsoid region's surface geometry, which is necessary to understand the wall interaction failure.</t>
         </is>
       </c>
     </row>
@@ -2082,16 +2080,16 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>3545</v>
+        <v>3940</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>[BUG] Wrong delxyz calculation in region_ellipsoid.cpp</t>
+          <t>Total energy changes when using the old version or the new version of LAMMPS</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/3545</t>
+          <t>https://github.com/lammps/lammps/issues/3940</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2112,11 +2110,11 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/3553</t>
+          <t>https://github.com/lammps/lammps/pull/3941</t>
         </is>
       </c>
       <c r="J30" s="2" t="n">
-        <v>3553</v>
+        <v>3941</v>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
@@ -2126,7 +2124,7 @@
       <c r="L30" s="3" t="inlineStr"/>
       <c r="M30" s="3" t="inlineStr">
         <is>
-          <t>The issue reports incorrect vector calculations in ellipsoid region surface code, involving mathematical formulas for contact distance vectors that are necessary to understand the bug.</t>
+          <t>The issue reports incorrect total energy values in molecular dynamics simulations, which is a scientific numerical correctness problem requiring understanding of LAMMPS energy calculations and neighbor list behavior.</t>
         </is>
       </c>
     </row>
@@ -2137,16 +2135,16 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>3925</v>
+        <v>4408</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>[BUG] fix wall/region with region style ellipsoid</t>
+          <t>[BUG] Fix deform leads to lost atoms</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/3925</t>
+          <t>https://github.com/lammps/lammps/issues/4408</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2167,11 +2165,11 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/3931</t>
+          <t>https://github.com/lammps/lammps/pull/4407</t>
         </is>
       </c>
       <c r="J31" s="2" t="n">
-        <v>3931</v>
+        <v>4407</v>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
@@ -2181,7 +2179,7 @@
       <c r="L31" s="3" t="inlineStr"/>
       <c r="M31" s="3" t="inlineStr">
         <is>
-          <t>The bug involves incorrect mathematical formulas for the ellipsoid region's surface geometry, which is necessary to understand the wall interaction failure.</t>
+          <t>The issue reports incorrect simulation behavior (lost atoms) in a Lennard-Jones fluid under shear flow, which is a domain-specific scientific correctness bug in molecular dynamics.</t>
         </is>
       </c>
     </row>
@@ -2192,16 +2190,16 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>3940</v>
+        <v>3929</v>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Total energy changes when using the old version or the new version of LAMMPS</t>
+          <t>[BUG] Dynamic groups do not update when run with KOKKOS.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/3940</t>
+          <t>https://github.com/lammps/lammps/issues/3929</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2217,16 +2215,17 @@
       <c r="G32" s="3" t="inlineStr"/>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>bug</t>
+          <t>bug
+kokkos_package</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/3941</t>
+          <t>https://github.com/lammps/lammps/pull/3930</t>
         </is>
       </c>
       <c r="J32" s="2" t="n">
-        <v>3941</v>
+        <v>3930</v>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
@@ -2236,27 +2235,27 @@
       <c r="L32" s="3" t="inlineStr"/>
       <c r="M32" s="3" t="inlineStr">
         <is>
-          <t>The issue reports incorrect total energy values in molecular dynamics simulations, which is a scientific numerical correctness problem requiring understanding of LAMMPS energy calculations and neighbor list behavior.</t>
+          <t>The bug involves dynamic groups based on a crystallographic (FCC) configuration criterion, which requires domain-specific scientific knowledge to understand the expected behavior.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>lammps/lammps</t>
+          <t>biopython/biopython</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>4408</v>
+        <v>4438</v>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>[BUG] Fix deform leads to lost atoms</t>
+          <t>Bio.Seq.transcribe does not evaluate to naturally explained DNA transcription</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/4408</t>
+          <t>https://github.com/biopython/biopython/issues/4438</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -2270,18 +2269,14 @@
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr"/>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>bug</t>
-        </is>
-      </c>
+      <c r="H33" s="3" t="inlineStr"/>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/4407</t>
+          <t>https://github.com/biopython/biopython/pull/4439</t>
         </is>
       </c>
       <c r="J33" s="2" t="n">
-        <v>4407</v>
+        <v>4439</v>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
@@ -2291,27 +2286,27 @@
       <c r="L33" s="3" t="inlineStr"/>
       <c r="M33" s="3" t="inlineStr">
         <is>
-          <t>The issue reports incorrect simulation behavior (lost atoms) in a Lennard-Jones fluid under shear flow, which is a domain-specific scientific correctness bug in molecular dynamics.</t>
+          <t>The issue concerns the biological definition of DNA transcription, specifically the distinction between template and coding strands, which requires domain-specific scientific knowledge to evaluate.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>lammps/lammps</t>
+          <t>biopython/biopython</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>3929</v>
+        <v>3842</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>[BUG] Dynamic groups do not update when run with KOKKOS.</t>
+          <t>formulas in biopython/Bio/SeqUtils/MeltingTemp.py  source code line 736-760 don't correspond to line 795-818</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/issues/3929</t>
+          <t>https://github.com/biopython/biopython/issues/3842</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2325,19 +2320,14 @@
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr"/>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>bug
-kokkos_package</t>
-        </is>
-      </c>
+      <c r="H34" s="3" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/lammps/lammps/pull/3930</t>
+          <t>https://github.com/biopython/biopython/pull/3846</t>
         </is>
       </c>
       <c r="J34" s="2" t="n">
-        <v>3930</v>
+        <v>3846</v>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
@@ -2347,7 +2337,7 @@
       <c r="L34" s="3" t="inlineStr"/>
       <c r="M34" s="3" t="inlineStr">
         <is>
-          <t>The bug involves dynamic groups based on a crystallographic (FCC) configuration criterion, which requires domain-specific scientific knowledge to understand the expected behavior.</t>
+          <t>The issue concerns inconsistencies between documented thermodynamic melting-temperature formulas and the salt-correction constants in the code, requiring domain-specific scientific knowledge of the equations.</t>
         </is>
       </c>
     </row>
@@ -2358,16 +2348,16 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>4438</v>
+        <v>3280</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Bio.Seq.transcribe does not evaluate to naturally explained DNA transcription</t>
+          <t>Discrepancies in Tm Values when using  MeltingTemp.Tm_NN(seq=, nn_table = MeltingTemp.R_DNA_NN1)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/biopython/biopython/issues/4438</t>
+          <t>https://github.com/biopython/biopython/issues/3280</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2384,11 +2374,11 @@
       <c r="H35" s="3" t="inlineStr"/>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/biopython/biopython/pull/4439</t>
+          <t>https://github.com/biopython/biopython/pull/3281</t>
         </is>
       </c>
       <c r="J35" s="2" t="n">
-        <v>4439</v>
+        <v>3281</v>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
@@ -2398,7 +2388,7 @@
       <c r="L35" s="3" t="inlineStr"/>
       <c r="M35" s="3" t="inlineStr">
         <is>
-          <t>The issue concerns the biological definition of DNA transcription, specifically the distinction between template and coding strands, which requires domain-specific scientific knowledge to evaluate.</t>
+          <t>The issue reports incorrect melting-temperature predictions from a nearest-neighbor thermodynamic model, requiring domain knowledge of nucleic acid thermodynamics and experimental conditions.</t>
         </is>
       </c>
     </row>
@@ -2409,16 +2399,16 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>3842</v>
+        <v>2280</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>formulas in biopython/Bio/SeqUtils/MeltingTemp.py  source code line 736-760 don't correspond to line 795-818</t>
+          <t>key err in DNA_TMM1 of Bio.SeqUtils for two NN pairs</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/biopython/biopython/issues/3842</t>
+          <t>https://github.com/biopython/biopython/issues/2280</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2435,11 +2425,11 @@
       <c r="H36" s="3" t="inlineStr"/>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/biopython/biopython/pull/3846</t>
+          <t>https://github.com/biopython/biopython/pull/2283</t>
         </is>
       </c>
       <c r="J36" s="2" t="n">
-        <v>3846</v>
+        <v>2283</v>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
@@ -2448,108 +2438,6 @@
       </c>
       <c r="L36" s="3" t="inlineStr"/>
       <c r="M36" s="3" t="inlineStr">
-        <is>
-          <t>The issue concerns inconsistencies between documented thermodynamic melting-temperature formulas and the salt-correction constants in the code, requiring domain-specific scientific knowledge of the equations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>biopython/biopython</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="n">
-        <v>3280</v>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>Discrepancies in Tm Values when using  MeltingTemp.Tm_NN(seq=, nn_table = MeltingTemp.R_DNA_NN1)</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>https://github.com/biopython/biopython/issues/3280</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr"/>
-      <c r="H37" s="3" t="inlineStr"/>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>https://github.com/biopython/biopython/pull/3281</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="n">
-        <v>3281</v>
-      </c>
-      <c r="K37" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L37" s="3" t="inlineStr"/>
-      <c r="M37" s="3" t="inlineStr">
-        <is>
-          <t>The issue reports incorrect melting-temperature predictions from a nearest-neighbor thermodynamic model, requiring domain knowledge of nucleic acid thermodynamics and experimental conditions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>biopython/biopython</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="n">
-        <v>2280</v>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>key err in DNA_TMM1 of Bio.SeqUtils for two NN pairs</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>https://github.com/biopython/biopython/issues/2280</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr"/>
-      <c r="H38" s="3" t="inlineStr"/>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>https://github.com/biopython/biopython/pull/2283</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="n">
-        <v>2283</v>
-      </c>
-      <c r="K38" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L38" s="3" t="inlineStr"/>
-      <c r="M38" s="3" t="inlineStr">
         <is>
           <t>The issue concerns incorrect DNA melting temperature calculations due to missing terminal mismatch nearest-neighbor thermodynamic parameters, requiring domain-specific knowledge of the Tm_NN model.</t>
         </is>
@@ -2598,11 +2486,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>91.9%</t>
+          <t>91.4%</t>
         </is>
       </c>
     </row>
@@ -2617,18 +2505,18 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.6%</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B4" s="1" t="n">
-        <v>37</v>
+      <c r="B4" t="n">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>